<commit_message>
Refresh screenshots, sample workbook and website
The sample workbook now has a styled, frozen header row, currency
columns, a bold totals row and a revenue chart on the Summary sheet. All
README screenshots are regenerated with the formatting toolbar, plus new
Charts and Formatting screenshots, and the website's showcase and
feature cards cover charts and styling.
</commit_message>
<xml_diff>
--- a/samples/sales.xlsx
+++ b/samples/sales.xlsx
@@ -111,10 +111,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -122,16 +123,38 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF15803D"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -139,13 +162,28 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -153,6 +191,156 @@
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:lang val="en-US"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>Revenue by region</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:layout/>
+    </c:title>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Summary!$B$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Revenue</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:cat>
+            <c:strRef>
+              <c:f>Summary!$A$2:$A$5</c:f>
+              <c:strCache>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>West</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>East</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>North</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>South</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Summary!$B$2:$B$5</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:axId val="50010001"/>
+        <c:axId val="50010002"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="50010001"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:axPos val="b"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="50010002"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="50010002"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:axPos val="l"/>
+        <c:majorGridlines/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="50010001"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:layout/>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+  </c:chart>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>533400</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -455,31 +643,31 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
     </row>
@@ -487,7 +675,7 @@
       <c r="A2">
         <v>1001</v>
       </c>
-      <c r="B2" s="1">
+      <c r="B2" s="2">
         <v>45295</v>
       </c>
       <c r="C2" t="s">
@@ -502,12 +690,12 @@
       <c r="F2">
         <v>9</v>
       </c>
-      <c r="G2">
+      <c r="G2" s="3">
         <v>3.5</v>
       </c>
-      <c r="H2">
+      <c r="H2" s="3" t="str">
         <f>F2*G2</f>
-        <v>31.5</v>
+        <v>$31.50</v>
       </c>
       <c r="I2" t="s">
         <v>12</v>
@@ -517,7 +705,7 @@
       <c r="A3">
         <v>1002</v>
       </c>
-      <c r="B3" s="1">
+      <c r="B3" s="2">
         <v>45301</v>
       </c>
       <c r="C3" t="s">
@@ -532,12 +720,12 @@
       <c r="F3">
         <v>8</v>
       </c>
-      <c r="G3">
+      <c r="G3" s="3">
         <v>42</v>
       </c>
-      <c r="H3">
+      <c r="H3" s="3" t="str">
         <f>F3*G3</f>
-        <v>336</v>
+        <v>$336.00</v>
       </c>
       <c r="I3" t="s">
         <v>16</v>
@@ -547,7 +735,7 @@
       <c r="A4">
         <v>1003</v>
       </c>
-      <c r="B4" s="1">
+      <c r="B4" s="2">
         <v>45312</v>
       </c>
       <c r="C4" t="s">
@@ -562,12 +750,12 @@
       <c r="F4">
         <v>14</v>
       </c>
-      <c r="G4">
+      <c r="G4" s="3">
         <v>120</v>
       </c>
-      <c r="H4">
+      <c r="H4" s="3" t="str">
         <f>F4*G4</f>
-        <v>1680</v>
+        <v>$1,680.00</v>
       </c>
       <c r="I4" t="s">
         <v>18</v>
@@ -577,7 +765,7 @@
       <c r="A5">
         <v>1004</v>
       </c>
-      <c r="B5" s="1">
+      <c r="B5" s="2">
         <v>45316</v>
       </c>
       <c r="C5" t="s">
@@ -592,12 +780,12 @@
       <c r="F5">
         <v>30</v>
       </c>
-      <c r="G5">
+      <c r="G5" s="3">
         <v>7.25</v>
       </c>
-      <c r="H5">
+      <c r="H5" s="3" t="str">
         <f>F5*G5</f>
-        <v>217.5</v>
+        <v>$217.50</v>
       </c>
       <c r="I5" t="s">
         <v>12</v>
@@ -607,7 +795,7 @@
       <c r="A6">
         <v>1005</v>
       </c>
-      <c r="B6" s="1">
+      <c r="B6" s="2">
         <v>45325</v>
       </c>
       <c r="C6" t="s">
@@ -622,12 +810,12 @@
       <c r="F6">
         <v>36</v>
       </c>
-      <c r="G6">
+      <c r="G6" s="3">
         <v>42</v>
       </c>
-      <c r="H6">
+      <c r="H6" s="3" t="str">
         <f>F6*G6</f>
-        <v>1512</v>
+        <v>$1,512.00</v>
       </c>
       <c r="I6" t="s">
         <v>16</v>
@@ -637,7 +825,7 @@
       <c r="A7">
         <v>1006</v>
       </c>
-      <c r="B7" s="1">
+      <c r="B7" s="2">
         <v>45330</v>
       </c>
       <c r="C7" t="s">
@@ -652,12 +840,12 @@
       <c r="F7">
         <v>25</v>
       </c>
-      <c r="G7">
+      <c r="G7" s="3">
         <v>120</v>
       </c>
-      <c r="H7">
+      <c r="H7" s="3" t="str">
         <f>F7*G7</f>
-        <v>3000</v>
+        <v>$3,000.00</v>
       </c>
       <c r="I7" t="s">
         <v>16</v>
@@ -667,7 +855,7 @@
       <c r="A8">
         <v>1007</v>
       </c>
-      <c r="B8" s="1">
+      <c r="B8" s="2">
         <v>45336</v>
       </c>
       <c r="C8" t="s">
@@ -682,12 +870,12 @@
       <c r="F8">
         <v>4</v>
       </c>
-      <c r="G8">
+      <c r="G8" s="3">
         <v>3.5</v>
       </c>
-      <c r="H8">
+      <c r="H8" s="3" t="str">
         <f>F8*G8</f>
-        <v>14</v>
+        <v>$14.00</v>
       </c>
       <c r="I8" t="s">
         <v>18</v>
@@ -697,7 +885,7 @@
       <c r="A9">
         <v>1008</v>
       </c>
-      <c r="B9" s="1">
+      <c r="B9" s="2">
         <v>45346</v>
       </c>
       <c r="C9" t="s">
@@ -712,12 +900,12 @@
       <c r="F9">
         <v>38</v>
       </c>
-      <c r="G9">
+      <c r="G9" s="3">
         <v>3.5</v>
       </c>
-      <c r="H9">
+      <c r="H9" s="3" t="str">
         <f>F9*G9</f>
-        <v>133</v>
+        <v>$133.00</v>
       </c>
       <c r="I9" t="s">
         <v>12</v>
@@ -727,7 +915,7 @@
       <c r="A10">
         <v>1009</v>
       </c>
-      <c r="B10" s="1">
+      <c r="B10" s="2">
         <v>45353</v>
       </c>
       <c r="C10" t="s">
@@ -742,12 +930,12 @@
       <c r="F10">
         <v>22</v>
       </c>
-      <c r="G10">
+      <c r="G10" s="3">
         <v>3.5</v>
       </c>
-      <c r="H10">
+      <c r="H10" s="3" t="str">
         <f>F10*G10</f>
-        <v>77</v>
+        <v>$77.00</v>
       </c>
       <c r="I10" t="s">
         <v>12</v>
@@ -757,7 +945,7 @@
       <c r="A11">
         <v>1010</v>
       </c>
-      <c r="B11" s="1">
+      <c r="B11" s="2">
         <v>45361</v>
       </c>
       <c r="C11" t="s">
@@ -772,12 +960,12 @@
       <c r="F11">
         <v>17</v>
       </c>
-      <c r="G11">
+      <c r="G11" s="3">
         <v>7.25</v>
       </c>
-      <c r="H11">
+      <c r="H11" s="3" t="str">
         <f>F11*G11</f>
-        <v>123.25</v>
+        <v>$123.25</v>
       </c>
       <c r="I11" t="s">
         <v>12</v>
@@ -787,7 +975,7 @@
       <c r="A12">
         <v>1011</v>
       </c>
-      <c r="B12" s="1">
+      <c r="B12" s="2">
         <v>45366</v>
       </c>
       <c r="C12" t="s">
@@ -802,12 +990,12 @@
       <c r="F12">
         <v>27</v>
       </c>
-      <c r="G12">
+      <c r="G12" s="3">
         <v>120</v>
       </c>
-      <c r="H12">
+      <c r="H12" s="3" t="str">
         <f>F12*G12</f>
-        <v>3240</v>
+        <v>$3,240.00</v>
       </c>
       <c r="I12" t="s">
         <v>12</v>
@@ -817,7 +1005,7 @@
       <c r="A13">
         <v>1012</v>
       </c>
-      <c r="B13" s="1">
+      <c r="B13" s="2">
         <v>45375</v>
       </c>
       <c r="C13" t="s">
@@ -832,12 +1020,12 @@
       <c r="F13">
         <v>25</v>
       </c>
-      <c r="G13">
+      <c r="G13" s="3">
         <v>7.25</v>
       </c>
-      <c r="H13">
+      <c r="H13" s="3" t="str">
         <f>F13*G13</f>
-        <v>181.25</v>
+        <v>$181.25</v>
       </c>
       <c r="I13" t="s">
         <v>12</v>
@@ -847,7 +1035,7 @@
       <c r="A14">
         <v>1013</v>
       </c>
-      <c r="B14" s="1">
+      <c r="B14" s="2">
         <v>45381</v>
       </c>
       <c r="C14" t="s">
@@ -862,12 +1050,12 @@
       <c r="F14">
         <v>24</v>
       </c>
-      <c r="G14">
+      <c r="G14" s="3">
         <v>3.5</v>
       </c>
-      <c r="H14">
+      <c r="H14" s="3" t="str">
         <f>F14*G14</f>
-        <v>84</v>
+        <v>$84.00</v>
       </c>
       <c r="I14" t="s">
         <v>12</v>
@@ -877,7 +1065,7 @@
       <c r="A15">
         <v>1014</v>
       </c>
-      <c r="B15" s="1">
+      <c r="B15" s="2">
         <v>45388</v>
       </c>
       <c r="C15" t="s">
@@ -892,12 +1080,12 @@
       <c r="F15">
         <v>26</v>
       </c>
-      <c r="G15">
+      <c r="G15" s="3">
         <v>3.5</v>
       </c>
-      <c r="H15">
+      <c r="H15" s="3" t="str">
         <f>F15*G15</f>
-        <v>91</v>
+        <v>$91.00</v>
       </c>
       <c r="I15" t="s">
         <v>12</v>
@@ -907,7 +1095,7 @@
       <c r="A16">
         <v>1015</v>
       </c>
-      <c r="B16" s="1">
+      <c r="B16" s="2">
         <v>45395</v>
       </c>
       <c r="C16" t="s">
@@ -922,12 +1110,12 @@
       <c r="F16">
         <v>14</v>
       </c>
-      <c r="G16">
+      <c r="G16" s="3">
         <v>42</v>
       </c>
-      <c r="H16">
+      <c r="H16" s="3" t="str">
         <f>F16*G16</f>
-        <v>588</v>
+        <v>$588.00</v>
       </c>
       <c r="I16" t="s">
         <v>12</v>
@@ -937,7 +1125,7 @@
       <c r="A17">
         <v>1016</v>
       </c>
-      <c r="B17" s="1">
+      <c r="B17" s="2">
         <v>45403</v>
       </c>
       <c r="C17" t="s">
@@ -952,12 +1140,12 @@
       <c r="F17">
         <v>25</v>
       </c>
-      <c r="G17">
+      <c r="G17" s="3">
         <v>120</v>
       </c>
-      <c r="H17">
+      <c r="H17" s="3" t="str">
         <f>F17*G17</f>
-        <v>3000</v>
+        <v>$3,000.00</v>
       </c>
       <c r="I17" t="s">
         <v>12</v>
@@ -967,7 +1155,7 @@
       <c r="A18">
         <v>1017</v>
       </c>
-      <c r="B18" s="1">
+      <c r="B18" s="2">
         <v>45408</v>
       </c>
       <c r="C18" t="s">
@@ -982,12 +1170,12 @@
       <c r="F18">
         <v>35</v>
       </c>
-      <c r="G18">
+      <c r="G18" s="3">
         <v>3.5</v>
       </c>
-      <c r="H18">
+      <c r="H18" s="3" t="str">
         <f>F18*G18</f>
-        <v>122.5</v>
+        <v>$122.50</v>
       </c>
       <c r="I18" t="s">
         <v>12</v>
@@ -997,7 +1185,7 @@
       <c r="A19">
         <v>1018</v>
       </c>
-      <c r="B19" s="1">
+      <c r="B19" s="2">
         <v>45413</v>
       </c>
       <c r="C19" t="s">
@@ -1012,12 +1200,12 @@
       <c r="F19">
         <v>19</v>
       </c>
-      <c r="G19">
+      <c r="G19" s="3">
         <v>19.99</v>
       </c>
-      <c r="H19">
+      <c r="H19" s="3" t="str">
         <f>F19*G19</f>
-        <v>379.81</v>
+        <v>$379.81</v>
       </c>
       <c r="I19" t="s">
         <v>16</v>
@@ -1027,7 +1215,7 @@
       <c r="A20">
         <v>1019</v>
       </c>
-      <c r="B20" s="1">
+      <c r="B20" s="2">
         <v>45422</v>
       </c>
       <c r="C20" t="s">
@@ -1042,12 +1230,12 @@
       <c r="F20">
         <v>34</v>
       </c>
-      <c r="G20">
+      <c r="G20" s="3">
         <v>7.25</v>
       </c>
-      <c r="H20">
+      <c r="H20" s="3" t="str">
         <f>F20*G20</f>
-        <v>246.5</v>
+        <v>$246.50</v>
       </c>
       <c r="I20" t="s">
         <v>16</v>
@@ -1057,7 +1245,7 @@
       <c r="A21">
         <v>1020</v>
       </c>
-      <c r="B21" s="1">
+      <c r="B21" s="2">
         <v>45429</v>
       </c>
       <c r="C21" t="s">
@@ -1072,12 +1260,12 @@
       <c r="F21">
         <v>22</v>
       </c>
-      <c r="G21">
+      <c r="G21" s="3">
         <v>42</v>
       </c>
-      <c r="H21">
+      <c r="H21" s="3" t="str">
         <f>F21*G21</f>
-        <v>924</v>
+        <v>$924.00</v>
       </c>
       <c r="I21" t="s">
         <v>16</v>
@@ -1087,7 +1275,7 @@
       <c r="A22">
         <v>1021</v>
       </c>
-      <c r="B22" s="1">
+      <c r="B22" s="2">
         <v>45435</v>
       </c>
       <c r="C22" t="s">
@@ -1102,12 +1290,12 @@
       <c r="F22">
         <v>6</v>
       </c>
-      <c r="G22">
+      <c r="G22" s="3">
         <v>42</v>
       </c>
-      <c r="H22">
+      <c r="H22" s="3" t="str">
         <f>F22*G22</f>
-        <v>252</v>
+        <v>$252.00</v>
       </c>
       <c r="I22" t="s">
         <v>12</v>
@@ -1117,7 +1305,7 @@
       <c r="A23">
         <v>1022</v>
       </c>
-      <c r="B23" s="1">
+      <c r="B23" s="2">
         <v>45441</v>
       </c>
       <c r="C23" t="s">
@@ -1132,12 +1320,12 @@
       <c r="F23">
         <v>17</v>
       </c>
-      <c r="G23">
+      <c r="G23" s="3">
         <v>19.99</v>
       </c>
-      <c r="H23">
+      <c r="H23" s="3" t="str">
         <f>F23*G23</f>
-        <v>339.83</v>
+        <v>$339.83</v>
       </c>
       <c r="I23" t="s">
         <v>16</v>
@@ -1147,7 +1335,7 @@
       <c r="A24">
         <v>1023</v>
       </c>
-      <c r="B24" s="1">
+      <c r="B24" s="2">
         <v>45449</v>
       </c>
       <c r="C24" t="s">
@@ -1162,12 +1350,12 @@
       <c r="F24">
         <v>31</v>
       </c>
-      <c r="G24">
+      <c r="G24" s="3">
         <v>7.25</v>
       </c>
-      <c r="H24">
+      <c r="H24" s="3" t="str">
         <f>F24*G24</f>
-        <v>224.75</v>
+        <v>$224.75</v>
       </c>
       <c r="I24" t="s">
         <v>12</v>
@@ -1177,7 +1365,7 @@
       <c r="A25">
         <v>1024</v>
       </c>
-      <c r="B25" s="1">
+      <c r="B25" s="2">
         <v>45458</v>
       </c>
       <c r="C25" t="s">
@@ -1192,12 +1380,12 @@
       <c r="F25">
         <v>25</v>
       </c>
-      <c r="G25">
+      <c r="G25" s="3">
         <v>3.5</v>
       </c>
-      <c r="H25">
+      <c r="H25" s="3" t="str">
         <f>F25*G25</f>
-        <v>87.5</v>
+        <v>$87.50</v>
       </c>
       <c r="I25" t="s">
         <v>18</v>
@@ -1207,7 +1395,7 @@
       <c r="A26">
         <v>1025</v>
       </c>
-      <c r="B26" s="1">
+      <c r="B26" s="2">
         <v>45463</v>
       </c>
       <c r="C26" t="s">
@@ -1222,12 +1410,12 @@
       <c r="F26">
         <v>25</v>
       </c>
-      <c r="G26">
+      <c r="G26" s="3">
         <v>42</v>
       </c>
-      <c r="H26">
+      <c r="H26" s="3" t="str">
         <f>F26*G26</f>
-        <v>1050</v>
+        <v>$1,050.00</v>
       </c>
       <c r="I26" t="s">
         <v>18</v>
@@ -1237,7 +1425,7 @@
       <c r="A27">
         <v>1026</v>
       </c>
-      <c r="B27" s="1">
+      <c r="B27" s="2">
         <v>45471</v>
       </c>
       <c r="C27" t="s">
@@ -1252,12 +1440,12 @@
       <c r="F27">
         <v>34</v>
       </c>
-      <c r="G27">
+      <c r="G27" s="3">
         <v>42</v>
       </c>
-      <c r="H27">
+      <c r="H27" s="3" t="str">
         <f>F27*G27</f>
-        <v>1428</v>
+        <v>$1,428.00</v>
       </c>
       <c r="I27" t="s">
         <v>12</v>
@@ -1267,7 +1455,7 @@
       <c r="A28">
         <v>1027</v>
       </c>
-      <c r="B28" s="1">
+      <c r="B28" s="2">
         <v>45476</v>
       </c>
       <c r="C28" t="s">
@@ -1282,12 +1470,12 @@
       <c r="F28">
         <v>32</v>
       </c>
-      <c r="G28">
+      <c r="G28" s="3">
         <v>120</v>
       </c>
-      <c r="H28">
+      <c r="H28" s="3" t="str">
         <f>F28*G28</f>
-        <v>3840</v>
+        <v>$3,840.00</v>
       </c>
       <c r="I28" t="s">
         <v>12</v>
@@ -1297,7 +1485,7 @@
       <c r="A29">
         <v>1028</v>
       </c>
-      <c r="B29" s="1">
+      <c r="B29" s="2">
         <v>45487</v>
       </c>
       <c r="C29" t="s">
@@ -1312,12 +1500,12 @@
       <c r="F29">
         <v>16</v>
       </c>
-      <c r="G29">
+      <c r="G29" s="3">
         <v>19.99</v>
       </c>
-      <c r="H29">
+      <c r="H29" s="3" t="str">
         <f>F29*G29</f>
-        <v>319.84</v>
+        <v>$319.84</v>
       </c>
       <c r="I29" t="s">
         <v>12</v>
@@ -1327,7 +1515,7 @@
       <c r="A30">
         <v>1029</v>
       </c>
-      <c r="B30" s="1">
+      <c r="B30" s="2">
         <v>45494</v>
       </c>
       <c r="C30" t="s">
@@ -1342,12 +1530,12 @@
       <c r="F30">
         <v>23</v>
       </c>
-      <c r="G30">
+      <c r="G30" s="3">
         <v>120</v>
       </c>
-      <c r="H30">
+      <c r="H30" s="3" t="str">
         <f>F30*G30</f>
-        <v>2760</v>
+        <v>$2,760.00</v>
       </c>
       <c r="I30" t="s">
         <v>18</v>
@@ -1357,7 +1545,7 @@
       <c r="A31">
         <v>1030</v>
       </c>
-      <c r="B31" s="1">
+      <c r="B31" s="2">
         <v>45498</v>
       </c>
       <c r="C31" t="s">
@@ -1372,12 +1560,12 @@
       <c r="F31">
         <v>3</v>
       </c>
-      <c r="G31">
+      <c r="G31" s="3">
         <v>120</v>
       </c>
-      <c r="H31">
+      <c r="H31" s="3" t="str">
         <f>F31*G31</f>
-        <v>360</v>
+        <v>$360.00</v>
       </c>
       <c r="I31" t="s">
         <v>16</v>
@@ -1387,7 +1575,7 @@
       <c r="A32">
         <v>1031</v>
       </c>
-      <c r="B32" s="1">
+      <c r="B32" s="2">
         <v>45507</v>
       </c>
       <c r="C32" t="s">
@@ -1402,12 +1590,12 @@
       <c r="F32">
         <v>19</v>
       </c>
-      <c r="G32">
+      <c r="G32" s="3">
         <v>19.99</v>
       </c>
-      <c r="H32">
+      <c r="H32" s="3" t="str">
         <f>F32*G32</f>
-        <v>379.81</v>
+        <v>$379.81</v>
       </c>
       <c r="I32" t="s">
         <v>18</v>
@@ -1417,7 +1605,7 @@
       <c r="A33">
         <v>1032</v>
       </c>
-      <c r="B33" s="1">
+      <c r="B33" s="2">
         <v>45514</v>
       </c>
       <c r="C33" t="s">
@@ -1432,12 +1620,12 @@
       <c r="F33">
         <v>9</v>
       </c>
-      <c r="G33">
+      <c r="G33" s="3">
         <v>120</v>
       </c>
-      <c r="H33">
+      <c r="H33" s="3" t="str">
         <f>F33*G33</f>
-        <v>1080</v>
+        <v>$1,080.00</v>
       </c>
       <c r="I33" t="s">
         <v>18</v>
@@ -1447,7 +1635,7 @@
       <c r="A34">
         <v>1033</v>
       </c>
-      <c r="B34" s="1">
+      <c r="B34" s="2">
         <v>45519</v>
       </c>
       <c r="C34" t="s">
@@ -1462,12 +1650,12 @@
       <c r="F34">
         <v>26</v>
       </c>
-      <c r="G34">
+      <c r="G34" s="3">
         <v>7.25</v>
       </c>
-      <c r="H34">
+      <c r="H34" s="3" t="str">
         <f>F34*G34</f>
-        <v>188.5</v>
+        <v>$188.50</v>
       </c>
       <c r="I34" t="s">
         <v>12</v>
@@ -1477,7 +1665,7 @@
       <c r="A35">
         <v>1034</v>
       </c>
-      <c r="B35" s="1">
+      <c r="B35" s="2">
         <v>45528</v>
       </c>
       <c r="C35" t="s">
@@ -1492,12 +1680,12 @@
       <c r="F35">
         <v>13</v>
       </c>
-      <c r="G35">
+      <c r="G35" s="3">
         <v>42</v>
       </c>
-      <c r="H35">
+      <c r="H35" s="3" t="str">
         <f>F35*G35</f>
-        <v>546</v>
+        <v>$546.00</v>
       </c>
       <c r="I35" t="s">
         <v>16</v>
@@ -1507,7 +1695,7 @@
       <c r="A36">
         <v>1035</v>
       </c>
-      <c r="B36" s="1">
+      <c r="B36" s="2">
         <v>45533</v>
       </c>
       <c r="C36" t="s">
@@ -1522,12 +1710,12 @@
       <c r="F36">
         <v>20</v>
       </c>
-      <c r="G36">
+      <c r="G36" s="3">
         <v>7.25</v>
       </c>
-      <c r="H36">
+      <c r="H36" s="3" t="str">
         <f>F36*G36</f>
-        <v>145</v>
+        <v>$145.00</v>
       </c>
       <c r="I36" t="s">
         <v>12</v>
@@ -1537,7 +1725,7 @@
       <c r="A37">
         <v>1036</v>
       </c>
-      <c r="B37" s="1">
+      <c r="B37" s="2">
         <v>45541</v>
       </c>
       <c r="C37" t="s">
@@ -1552,12 +1740,12 @@
       <c r="F37">
         <v>1</v>
       </c>
-      <c r="G37">
+      <c r="G37" s="3">
         <v>120</v>
       </c>
-      <c r="H37">
+      <c r="H37" s="3" t="str">
         <f>F37*G37</f>
-        <v>120</v>
+        <v>$120.00</v>
       </c>
       <c r="I37" t="s">
         <v>16</v>
@@ -1567,7 +1755,7 @@
       <c r="A38">
         <v>1037</v>
       </c>
-      <c r="B38" s="1">
+      <c r="B38" s="2">
         <v>45548</v>
       </c>
       <c r="C38" t="s">
@@ -1582,12 +1770,12 @@
       <c r="F38">
         <v>27</v>
       </c>
-      <c r="G38">
+      <c r="G38" s="3">
         <v>120</v>
       </c>
-      <c r="H38">
+      <c r="H38" s="3" t="str">
         <f>F38*G38</f>
-        <v>3240</v>
+        <v>$3,240.00</v>
       </c>
       <c r="I38" t="s">
         <v>12</v>
@@ -1597,7 +1785,7 @@
       <c r="A39">
         <v>1038</v>
       </c>
-      <c r="B39" s="1">
+      <c r="B39" s="2">
         <v>45554</v>
       </c>
       <c r="C39" t="s">
@@ -1612,12 +1800,12 @@
       <c r="F39">
         <v>1</v>
       </c>
-      <c r="G39">
+      <c r="G39" s="3">
         <v>42</v>
       </c>
-      <c r="H39">
+      <c r="H39" s="3" t="str">
         <f>F39*G39</f>
-        <v>42</v>
+        <v>$42.00</v>
       </c>
       <c r="I39" t="s">
         <v>12</v>
@@ -1627,7 +1815,7 @@
       <c r="A40">
         <v>1039</v>
       </c>
-      <c r="B40" s="1">
+      <c r="B40" s="2">
         <v>45560</v>
       </c>
       <c r="C40" t="s">
@@ -1642,12 +1830,12 @@
       <c r="F40">
         <v>20</v>
       </c>
-      <c r="G40">
+      <c r="G40" s="3">
         <v>7.25</v>
       </c>
-      <c r="H40">
+      <c r="H40" s="3" t="str">
         <f>F40*G40</f>
-        <v>145</v>
+        <v>$145.00</v>
       </c>
       <c r="I40" t="s">
         <v>12</v>
@@ -1657,7 +1845,7 @@
       <c r="A41">
         <v>1040</v>
       </c>
-      <c r="B41" s="1">
+      <c r="B41" s="2">
         <v>45569</v>
       </c>
       <c r="C41" t="s">
@@ -1672,12 +1860,12 @@
       <c r="F41">
         <v>29</v>
       </c>
-      <c r="G41">
+      <c r="G41" s="3">
         <v>19.99</v>
       </c>
-      <c r="H41">
+      <c r="H41" s="3" t="str">
         <f>F41*G41</f>
-        <v>579.71</v>
+        <v>$579.71</v>
       </c>
       <c r="I41" t="s">
         <v>12</v>
@@ -1687,7 +1875,7 @@
       <c r="A42">
         <v>1041</v>
       </c>
-      <c r="B42" s="1">
+      <c r="B42" s="2">
         <v>45578</v>
       </c>
       <c r="C42" t="s">
@@ -1702,12 +1890,12 @@
       <c r="F42">
         <v>18</v>
       </c>
-      <c r="G42">
+      <c r="G42" s="3">
         <v>3.5</v>
       </c>
-      <c r="H42">
+      <c r="H42" s="3" t="str">
         <f>F42*G42</f>
-        <v>63</v>
+        <v>$63.00</v>
       </c>
       <c r="I42" t="s">
         <v>12</v>
@@ -1717,7 +1905,7 @@
       <c r="A43">
         <v>1042</v>
       </c>
-      <c r="B43" s="1">
+      <c r="B43" s="2">
         <v>45583</v>
       </c>
       <c r="C43" t="s">
@@ -1732,12 +1920,12 @@
       <c r="F43">
         <v>1</v>
       </c>
-      <c r="G43">
+      <c r="G43" s="3">
         <v>19.99</v>
       </c>
-      <c r="H43">
+      <c r="H43" s="3" t="str">
         <f>F43*G43</f>
-        <v>19.99</v>
+        <v>$19.99</v>
       </c>
       <c r="I43" t="s">
         <v>18</v>
@@ -1747,7 +1935,7 @@
       <c r="A44">
         <v>1043</v>
       </c>
-      <c r="B44" s="1">
+      <c r="B44" s="2">
         <v>45592</v>
       </c>
       <c r="C44" t="s">
@@ -1762,12 +1950,12 @@
       <c r="F44">
         <v>8</v>
       </c>
-      <c r="G44">
+      <c r="G44" s="3">
         <v>7.25</v>
       </c>
-      <c r="H44">
+      <c r="H44" s="3" t="str">
         <f>F44*G44</f>
-        <v>58</v>
+        <v>$58.00</v>
       </c>
       <c r="I44" t="s">
         <v>12</v>
@@ -1777,7 +1965,7 @@
       <c r="A45">
         <v>1044</v>
       </c>
-      <c r="B45" s="1">
+      <c r="B45" s="2">
         <v>45596</v>
       </c>
       <c r="C45" t="s">
@@ -1792,12 +1980,12 @@
       <c r="F45">
         <v>36</v>
       </c>
-      <c r="G45">
+      <c r="G45" s="3">
         <v>7.25</v>
       </c>
-      <c r="H45">
+      <c r="H45" s="3" t="str">
         <f>F45*G45</f>
-        <v>261</v>
+        <v>$261.00</v>
       </c>
       <c r="I45" t="s">
         <v>12</v>
@@ -1807,7 +1995,7 @@
       <c r="A46">
         <v>1045</v>
       </c>
-      <c r="B46" s="1">
+      <c r="B46" s="2">
         <v>45604</v>
       </c>
       <c r="C46" t="s">
@@ -1822,12 +2010,12 @@
       <c r="F46">
         <v>29</v>
       </c>
-      <c r="G46">
+      <c r="G46" s="3">
         <v>7.25</v>
       </c>
-      <c r="H46">
+      <c r="H46" s="3" t="str">
         <f>F46*G46</f>
-        <v>210.25</v>
+        <v>$210.25</v>
       </c>
       <c r="I46" t="s">
         <v>16</v>
@@ -1837,7 +2025,7 @@
       <c r="A47">
         <v>1046</v>
       </c>
-      <c r="B47" s="1">
+      <c r="B47" s="2">
         <v>45610</v>
       </c>
       <c r="C47" t="s">
@@ -1852,12 +2040,12 @@
       <c r="F47">
         <v>35</v>
       </c>
-      <c r="G47">
+      <c r="G47" s="3">
         <v>19.99</v>
       </c>
-      <c r="H47">
+      <c r="H47" s="3" t="str">
         <f>F47*G47</f>
-        <v>699.65</v>
+        <v>$699.65</v>
       </c>
       <c r="I47" t="s">
         <v>16</v>
@@ -1867,7 +2055,7 @@
       <c r="A48">
         <v>1047</v>
       </c>
-      <c r="B48" s="1">
+      <c r="B48" s="2">
         <v>45619</v>
       </c>
       <c r="C48" t="s">
@@ -1882,12 +2070,12 @@
       <c r="F48">
         <v>34</v>
       </c>
-      <c r="G48">
+      <c r="G48" s="3">
         <v>3.5</v>
       </c>
-      <c r="H48">
+      <c r="H48" s="3" t="str">
         <f>F48*G48</f>
-        <v>119</v>
+        <v>$119.00</v>
       </c>
       <c r="I48" t="s">
         <v>18</v>
@@ -1897,7 +2085,7 @@
       <c r="A49">
         <v>1048</v>
       </c>
-      <c r="B49" s="1">
+      <c r="B49" s="2">
         <v>45623</v>
       </c>
       <c r="C49" t="s">
@@ -1912,12 +2100,12 @@
       <c r="F49">
         <v>25</v>
       </c>
-      <c r="G49">
+      <c r="G49" s="3">
         <v>19.99</v>
       </c>
-      <c r="H49">
+      <c r="H49" s="3" t="str">
         <f>F49*G49</f>
-        <v>499.75</v>
+        <v>$499.75</v>
       </c>
       <c r="I49" t="s">
         <v>16</v>
@@ -1939,16 +2127,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>28</v>
       </c>
     </row>
@@ -1956,85 +2144,85 @@
       <c r="A2" t="s">
         <v>9</v>
       </c>
-      <c r="B2">
+      <c r="B2" s="3" t="str">
         <f>SUMIF(Orders!C$2:C$49,A2,Orders!H$2:H$49)</f>
-        <v>9439.3</v>
+        <v>$9,439.30</v>
       </c>
       <c r="C2">
         <f>COUNTIF(Orders!C$2:C$49,A2)</f>
         <v>10</v>
       </c>
-      <c r="D2">
+      <c r="D2" s="3" t="str">
         <f>ROUND(B2/C2,2)</f>
-        <v>943.93</v>
+        <v>$943.93</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" t="s">
         <v>23</v>
       </c>
-      <c r="B3">
+      <c r="B3" s="3" t="str">
         <f>SUMIF(Orders!C$2:C$49,A3,Orders!H$2:H$49)</f>
-        <v>6570.89</v>
+        <v>$6,570.89</v>
       </c>
       <c r="C3">
         <f>COUNTIF(Orders!C$2:C$49,A3)</f>
         <v>11</v>
       </c>
-      <c r="D3">
+      <c r="D3" s="3" t="str">
         <f>ROUND(B3/C3,2)</f>
-        <v>597.35</v>
+        <v>$597.35</v>
       </c>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" t="s">
         <v>13</v>
       </c>
-      <c r="B4">
+      <c r="B4" s="3" t="str">
         <f>SUMIF(Orders!C$2:C$49,A4,Orders!H$2:H$49)</f>
-        <v>7837</v>
+        <v>$7,837.00</v>
       </c>
       <c r="C4">
         <f>COUNTIF(Orders!C$2:C$49,A4)</f>
         <v>15</v>
       </c>
-      <c r="D4">
+      <c r="D4" s="3" t="str">
         <f>ROUND(B4/C4,2)</f>
-        <v>522.47</v>
+        <v>$522.47</v>
       </c>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" t="s">
         <v>19</v>
       </c>
-      <c r="B5">
+      <c r="B5" s="3" t="str">
         <f>SUMIF(Orders!C$2:C$49,A5,Orders!H$2:H$49)</f>
-        <v>11192.7</v>
+        <v>$11,192.70</v>
       </c>
       <c r="C5">
         <f>COUNTIF(Orders!C$2:C$49,A5)</f>
         <v>12</v>
       </c>
-      <c r="D5">
+      <c r="D5" s="3" t="str">
         <f>ROUND(B5/C5,2)</f>
-        <v>932.73</v>
+        <v>$932.73</v>
       </c>
     </row>
     <row r="6" spans="1:4">
-      <c r="A6" t="s">
+      <c r="A6" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="B6">
+      <c r="B6" s="5" t="str">
         <f>SUM(B2:B5)</f>
-        <v>35039.89</v>
-      </c>
-      <c r="C6">
+        <v>$35,039.89</v>
+      </c>
+      <c r="C6" s="4">
         <f>SUM(C2:C5)</f>
         <v>48</v>
       </c>
-      <c r="D6">
+      <c r="D6" s="5" t="str">
         <f>ROUND(B6/C6,2)</f>
-        <v>730</v>
+        <v>$730.00</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -2048,5 +2236,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Refresh screenshots, sample workbook and website (#17)
The sample workbook now has a styled, frozen header row, currency
columns, a bold totals row and a revenue chart on the Summary sheet. All
README screenshots are regenerated with the formatting toolbar, plus new
Charts and Formatting screenshots, and the website's showcase and
feature cards cover charts and styling.
</commit_message>
<xml_diff>
--- a/samples/sales.xlsx
+++ b/samples/sales.xlsx
@@ -111,10 +111,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -122,16 +123,38 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF15803D"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -139,13 +162,28 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -153,6 +191,156 @@
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:lang val="en-US"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>Revenue by region</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:layout/>
+    </c:title>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Summary!$B$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Revenue</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:cat>
+            <c:strRef>
+              <c:f>Summary!$A$2:$A$5</c:f>
+              <c:strCache>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>West</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>East</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>North</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>South</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Summary!$B$2:$B$5</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:axId val="50010001"/>
+        <c:axId val="50010002"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="50010001"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:axPos val="b"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="50010002"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="50010002"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:axPos val="l"/>
+        <c:majorGridlines/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="50010001"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:layout/>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+  </c:chart>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>533400</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -455,31 +643,31 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
     </row>
@@ -487,7 +675,7 @@
       <c r="A2">
         <v>1001</v>
       </c>
-      <c r="B2" s="1">
+      <c r="B2" s="2">
         <v>45295</v>
       </c>
       <c r="C2" t="s">
@@ -502,12 +690,12 @@
       <c r="F2">
         <v>9</v>
       </c>
-      <c r="G2">
+      <c r="G2" s="3">
         <v>3.5</v>
       </c>
-      <c r="H2">
+      <c r="H2" s="3" t="str">
         <f>F2*G2</f>
-        <v>31.5</v>
+        <v>$31.50</v>
       </c>
       <c r="I2" t="s">
         <v>12</v>
@@ -517,7 +705,7 @@
       <c r="A3">
         <v>1002</v>
       </c>
-      <c r="B3" s="1">
+      <c r="B3" s="2">
         <v>45301</v>
       </c>
       <c r="C3" t="s">
@@ -532,12 +720,12 @@
       <c r="F3">
         <v>8</v>
       </c>
-      <c r="G3">
+      <c r="G3" s="3">
         <v>42</v>
       </c>
-      <c r="H3">
+      <c r="H3" s="3" t="str">
         <f>F3*G3</f>
-        <v>336</v>
+        <v>$336.00</v>
       </c>
       <c r="I3" t="s">
         <v>16</v>
@@ -547,7 +735,7 @@
       <c r="A4">
         <v>1003</v>
       </c>
-      <c r="B4" s="1">
+      <c r="B4" s="2">
         <v>45312</v>
       </c>
       <c r="C4" t="s">
@@ -562,12 +750,12 @@
       <c r="F4">
         <v>14</v>
       </c>
-      <c r="G4">
+      <c r="G4" s="3">
         <v>120</v>
       </c>
-      <c r="H4">
+      <c r="H4" s="3" t="str">
         <f>F4*G4</f>
-        <v>1680</v>
+        <v>$1,680.00</v>
       </c>
       <c r="I4" t="s">
         <v>18</v>
@@ -577,7 +765,7 @@
       <c r="A5">
         <v>1004</v>
       </c>
-      <c r="B5" s="1">
+      <c r="B5" s="2">
         <v>45316</v>
       </c>
       <c r="C5" t="s">
@@ -592,12 +780,12 @@
       <c r="F5">
         <v>30</v>
       </c>
-      <c r="G5">
+      <c r="G5" s="3">
         <v>7.25</v>
       </c>
-      <c r="H5">
+      <c r="H5" s="3" t="str">
         <f>F5*G5</f>
-        <v>217.5</v>
+        <v>$217.50</v>
       </c>
       <c r="I5" t="s">
         <v>12</v>
@@ -607,7 +795,7 @@
       <c r="A6">
         <v>1005</v>
       </c>
-      <c r="B6" s="1">
+      <c r="B6" s="2">
         <v>45325</v>
       </c>
       <c r="C6" t="s">
@@ -622,12 +810,12 @@
       <c r="F6">
         <v>36</v>
       </c>
-      <c r="G6">
+      <c r="G6" s="3">
         <v>42</v>
       </c>
-      <c r="H6">
+      <c r="H6" s="3" t="str">
         <f>F6*G6</f>
-        <v>1512</v>
+        <v>$1,512.00</v>
       </c>
       <c r="I6" t="s">
         <v>16</v>
@@ -637,7 +825,7 @@
       <c r="A7">
         <v>1006</v>
       </c>
-      <c r="B7" s="1">
+      <c r="B7" s="2">
         <v>45330</v>
       </c>
       <c r="C7" t="s">
@@ -652,12 +840,12 @@
       <c r="F7">
         <v>25</v>
       </c>
-      <c r="G7">
+      <c r="G7" s="3">
         <v>120</v>
       </c>
-      <c r="H7">
+      <c r="H7" s="3" t="str">
         <f>F7*G7</f>
-        <v>3000</v>
+        <v>$3,000.00</v>
       </c>
       <c r="I7" t="s">
         <v>16</v>
@@ -667,7 +855,7 @@
       <c r="A8">
         <v>1007</v>
       </c>
-      <c r="B8" s="1">
+      <c r="B8" s="2">
         <v>45336</v>
       </c>
       <c r="C8" t="s">
@@ -682,12 +870,12 @@
       <c r="F8">
         <v>4</v>
       </c>
-      <c r="G8">
+      <c r="G8" s="3">
         <v>3.5</v>
       </c>
-      <c r="H8">
+      <c r="H8" s="3" t="str">
         <f>F8*G8</f>
-        <v>14</v>
+        <v>$14.00</v>
       </c>
       <c r="I8" t="s">
         <v>18</v>
@@ -697,7 +885,7 @@
       <c r="A9">
         <v>1008</v>
       </c>
-      <c r="B9" s="1">
+      <c r="B9" s="2">
         <v>45346</v>
       </c>
       <c r="C9" t="s">
@@ -712,12 +900,12 @@
       <c r="F9">
         <v>38</v>
       </c>
-      <c r="G9">
+      <c r="G9" s="3">
         <v>3.5</v>
       </c>
-      <c r="H9">
+      <c r="H9" s="3" t="str">
         <f>F9*G9</f>
-        <v>133</v>
+        <v>$133.00</v>
       </c>
       <c r="I9" t="s">
         <v>12</v>
@@ -727,7 +915,7 @@
       <c r="A10">
         <v>1009</v>
       </c>
-      <c r="B10" s="1">
+      <c r="B10" s="2">
         <v>45353</v>
       </c>
       <c r="C10" t="s">
@@ -742,12 +930,12 @@
       <c r="F10">
         <v>22</v>
       </c>
-      <c r="G10">
+      <c r="G10" s="3">
         <v>3.5</v>
       </c>
-      <c r="H10">
+      <c r="H10" s="3" t="str">
         <f>F10*G10</f>
-        <v>77</v>
+        <v>$77.00</v>
       </c>
       <c r="I10" t="s">
         <v>12</v>
@@ -757,7 +945,7 @@
       <c r="A11">
         <v>1010</v>
       </c>
-      <c r="B11" s="1">
+      <c r="B11" s="2">
         <v>45361</v>
       </c>
       <c r="C11" t="s">
@@ -772,12 +960,12 @@
       <c r="F11">
         <v>17</v>
       </c>
-      <c r="G11">
+      <c r="G11" s="3">
         <v>7.25</v>
       </c>
-      <c r="H11">
+      <c r="H11" s="3" t="str">
         <f>F11*G11</f>
-        <v>123.25</v>
+        <v>$123.25</v>
       </c>
       <c r="I11" t="s">
         <v>12</v>
@@ -787,7 +975,7 @@
       <c r="A12">
         <v>1011</v>
       </c>
-      <c r="B12" s="1">
+      <c r="B12" s="2">
         <v>45366</v>
       </c>
       <c r="C12" t="s">
@@ -802,12 +990,12 @@
       <c r="F12">
         <v>27</v>
       </c>
-      <c r="G12">
+      <c r="G12" s="3">
         <v>120</v>
       </c>
-      <c r="H12">
+      <c r="H12" s="3" t="str">
         <f>F12*G12</f>
-        <v>3240</v>
+        <v>$3,240.00</v>
       </c>
       <c r="I12" t="s">
         <v>12</v>
@@ -817,7 +1005,7 @@
       <c r="A13">
         <v>1012</v>
       </c>
-      <c r="B13" s="1">
+      <c r="B13" s="2">
         <v>45375</v>
       </c>
       <c r="C13" t="s">
@@ -832,12 +1020,12 @@
       <c r="F13">
         <v>25</v>
       </c>
-      <c r="G13">
+      <c r="G13" s="3">
         <v>7.25</v>
       </c>
-      <c r="H13">
+      <c r="H13" s="3" t="str">
         <f>F13*G13</f>
-        <v>181.25</v>
+        <v>$181.25</v>
       </c>
       <c r="I13" t="s">
         <v>12</v>
@@ -847,7 +1035,7 @@
       <c r="A14">
         <v>1013</v>
       </c>
-      <c r="B14" s="1">
+      <c r="B14" s="2">
         <v>45381</v>
       </c>
       <c r="C14" t="s">
@@ -862,12 +1050,12 @@
       <c r="F14">
         <v>24</v>
       </c>
-      <c r="G14">
+      <c r="G14" s="3">
         <v>3.5</v>
       </c>
-      <c r="H14">
+      <c r="H14" s="3" t="str">
         <f>F14*G14</f>
-        <v>84</v>
+        <v>$84.00</v>
       </c>
       <c r="I14" t="s">
         <v>12</v>
@@ -877,7 +1065,7 @@
       <c r="A15">
         <v>1014</v>
       </c>
-      <c r="B15" s="1">
+      <c r="B15" s="2">
         <v>45388</v>
       </c>
       <c r="C15" t="s">
@@ -892,12 +1080,12 @@
       <c r="F15">
         <v>26</v>
       </c>
-      <c r="G15">
+      <c r="G15" s="3">
         <v>3.5</v>
       </c>
-      <c r="H15">
+      <c r="H15" s="3" t="str">
         <f>F15*G15</f>
-        <v>91</v>
+        <v>$91.00</v>
       </c>
       <c r="I15" t="s">
         <v>12</v>
@@ -907,7 +1095,7 @@
       <c r="A16">
         <v>1015</v>
       </c>
-      <c r="B16" s="1">
+      <c r="B16" s="2">
         <v>45395</v>
       </c>
       <c r="C16" t="s">
@@ -922,12 +1110,12 @@
       <c r="F16">
         <v>14</v>
       </c>
-      <c r="G16">
+      <c r="G16" s="3">
         <v>42</v>
       </c>
-      <c r="H16">
+      <c r="H16" s="3" t="str">
         <f>F16*G16</f>
-        <v>588</v>
+        <v>$588.00</v>
       </c>
       <c r="I16" t="s">
         <v>12</v>
@@ -937,7 +1125,7 @@
       <c r="A17">
         <v>1016</v>
       </c>
-      <c r="B17" s="1">
+      <c r="B17" s="2">
         <v>45403</v>
       </c>
       <c r="C17" t="s">
@@ -952,12 +1140,12 @@
       <c r="F17">
         <v>25</v>
       </c>
-      <c r="G17">
+      <c r="G17" s="3">
         <v>120</v>
       </c>
-      <c r="H17">
+      <c r="H17" s="3" t="str">
         <f>F17*G17</f>
-        <v>3000</v>
+        <v>$3,000.00</v>
       </c>
       <c r="I17" t="s">
         <v>12</v>
@@ -967,7 +1155,7 @@
       <c r="A18">
         <v>1017</v>
       </c>
-      <c r="B18" s="1">
+      <c r="B18" s="2">
         <v>45408</v>
       </c>
       <c r="C18" t="s">
@@ -982,12 +1170,12 @@
       <c r="F18">
         <v>35</v>
       </c>
-      <c r="G18">
+      <c r="G18" s="3">
         <v>3.5</v>
       </c>
-      <c r="H18">
+      <c r="H18" s="3" t="str">
         <f>F18*G18</f>
-        <v>122.5</v>
+        <v>$122.50</v>
       </c>
       <c r="I18" t="s">
         <v>12</v>
@@ -997,7 +1185,7 @@
       <c r="A19">
         <v>1018</v>
       </c>
-      <c r="B19" s="1">
+      <c r="B19" s="2">
         <v>45413</v>
       </c>
       <c r="C19" t="s">
@@ -1012,12 +1200,12 @@
       <c r="F19">
         <v>19</v>
       </c>
-      <c r="G19">
+      <c r="G19" s="3">
         <v>19.99</v>
       </c>
-      <c r="H19">
+      <c r="H19" s="3" t="str">
         <f>F19*G19</f>
-        <v>379.81</v>
+        <v>$379.81</v>
       </c>
       <c r="I19" t="s">
         <v>16</v>
@@ -1027,7 +1215,7 @@
       <c r="A20">
         <v>1019</v>
       </c>
-      <c r="B20" s="1">
+      <c r="B20" s="2">
         <v>45422</v>
       </c>
       <c r="C20" t="s">
@@ -1042,12 +1230,12 @@
       <c r="F20">
         <v>34</v>
       </c>
-      <c r="G20">
+      <c r="G20" s="3">
         <v>7.25</v>
       </c>
-      <c r="H20">
+      <c r="H20" s="3" t="str">
         <f>F20*G20</f>
-        <v>246.5</v>
+        <v>$246.50</v>
       </c>
       <c r="I20" t="s">
         <v>16</v>
@@ -1057,7 +1245,7 @@
       <c r="A21">
         <v>1020</v>
       </c>
-      <c r="B21" s="1">
+      <c r="B21" s="2">
         <v>45429</v>
       </c>
       <c r="C21" t="s">
@@ -1072,12 +1260,12 @@
       <c r="F21">
         <v>22</v>
       </c>
-      <c r="G21">
+      <c r="G21" s="3">
         <v>42</v>
       </c>
-      <c r="H21">
+      <c r="H21" s="3" t="str">
         <f>F21*G21</f>
-        <v>924</v>
+        <v>$924.00</v>
       </c>
       <c r="I21" t="s">
         <v>16</v>
@@ -1087,7 +1275,7 @@
       <c r="A22">
         <v>1021</v>
       </c>
-      <c r="B22" s="1">
+      <c r="B22" s="2">
         <v>45435</v>
       </c>
       <c r="C22" t="s">
@@ -1102,12 +1290,12 @@
       <c r="F22">
         <v>6</v>
       </c>
-      <c r="G22">
+      <c r="G22" s="3">
         <v>42</v>
       </c>
-      <c r="H22">
+      <c r="H22" s="3" t="str">
         <f>F22*G22</f>
-        <v>252</v>
+        <v>$252.00</v>
       </c>
       <c r="I22" t="s">
         <v>12</v>
@@ -1117,7 +1305,7 @@
       <c r="A23">
         <v>1022</v>
       </c>
-      <c r="B23" s="1">
+      <c r="B23" s="2">
         <v>45441</v>
       </c>
       <c r="C23" t="s">
@@ -1132,12 +1320,12 @@
       <c r="F23">
         <v>17</v>
       </c>
-      <c r="G23">
+      <c r="G23" s="3">
         <v>19.99</v>
       </c>
-      <c r="H23">
+      <c r="H23" s="3" t="str">
         <f>F23*G23</f>
-        <v>339.83</v>
+        <v>$339.83</v>
       </c>
       <c r="I23" t="s">
         <v>16</v>
@@ -1147,7 +1335,7 @@
       <c r="A24">
         <v>1023</v>
       </c>
-      <c r="B24" s="1">
+      <c r="B24" s="2">
         <v>45449</v>
       </c>
       <c r="C24" t="s">
@@ -1162,12 +1350,12 @@
       <c r="F24">
         <v>31</v>
       </c>
-      <c r="G24">
+      <c r="G24" s="3">
         <v>7.25</v>
       </c>
-      <c r="H24">
+      <c r="H24" s="3" t="str">
         <f>F24*G24</f>
-        <v>224.75</v>
+        <v>$224.75</v>
       </c>
       <c r="I24" t="s">
         <v>12</v>
@@ -1177,7 +1365,7 @@
       <c r="A25">
         <v>1024</v>
       </c>
-      <c r="B25" s="1">
+      <c r="B25" s="2">
         <v>45458</v>
       </c>
       <c r="C25" t="s">
@@ -1192,12 +1380,12 @@
       <c r="F25">
         <v>25</v>
       </c>
-      <c r="G25">
+      <c r="G25" s="3">
         <v>3.5</v>
       </c>
-      <c r="H25">
+      <c r="H25" s="3" t="str">
         <f>F25*G25</f>
-        <v>87.5</v>
+        <v>$87.50</v>
       </c>
       <c r="I25" t="s">
         <v>18</v>
@@ -1207,7 +1395,7 @@
       <c r="A26">
         <v>1025</v>
       </c>
-      <c r="B26" s="1">
+      <c r="B26" s="2">
         <v>45463</v>
       </c>
       <c r="C26" t="s">
@@ -1222,12 +1410,12 @@
       <c r="F26">
         <v>25</v>
       </c>
-      <c r="G26">
+      <c r="G26" s="3">
         <v>42</v>
       </c>
-      <c r="H26">
+      <c r="H26" s="3" t="str">
         <f>F26*G26</f>
-        <v>1050</v>
+        <v>$1,050.00</v>
       </c>
       <c r="I26" t="s">
         <v>18</v>
@@ -1237,7 +1425,7 @@
       <c r="A27">
         <v>1026</v>
       </c>
-      <c r="B27" s="1">
+      <c r="B27" s="2">
         <v>45471</v>
       </c>
       <c r="C27" t="s">
@@ -1252,12 +1440,12 @@
       <c r="F27">
         <v>34</v>
       </c>
-      <c r="G27">
+      <c r="G27" s="3">
         <v>42</v>
       </c>
-      <c r="H27">
+      <c r="H27" s="3" t="str">
         <f>F27*G27</f>
-        <v>1428</v>
+        <v>$1,428.00</v>
       </c>
       <c r="I27" t="s">
         <v>12</v>
@@ -1267,7 +1455,7 @@
       <c r="A28">
         <v>1027</v>
       </c>
-      <c r="B28" s="1">
+      <c r="B28" s="2">
         <v>45476</v>
       </c>
       <c r="C28" t="s">
@@ -1282,12 +1470,12 @@
       <c r="F28">
         <v>32</v>
       </c>
-      <c r="G28">
+      <c r="G28" s="3">
         <v>120</v>
       </c>
-      <c r="H28">
+      <c r="H28" s="3" t="str">
         <f>F28*G28</f>
-        <v>3840</v>
+        <v>$3,840.00</v>
       </c>
       <c r="I28" t="s">
         <v>12</v>
@@ -1297,7 +1485,7 @@
       <c r="A29">
         <v>1028</v>
       </c>
-      <c r="B29" s="1">
+      <c r="B29" s="2">
         <v>45487</v>
       </c>
       <c r="C29" t="s">
@@ -1312,12 +1500,12 @@
       <c r="F29">
         <v>16</v>
       </c>
-      <c r="G29">
+      <c r="G29" s="3">
         <v>19.99</v>
       </c>
-      <c r="H29">
+      <c r="H29" s="3" t="str">
         <f>F29*G29</f>
-        <v>319.84</v>
+        <v>$319.84</v>
       </c>
       <c r="I29" t="s">
         <v>12</v>
@@ -1327,7 +1515,7 @@
       <c r="A30">
         <v>1029</v>
       </c>
-      <c r="B30" s="1">
+      <c r="B30" s="2">
         <v>45494</v>
       </c>
       <c r="C30" t="s">
@@ -1342,12 +1530,12 @@
       <c r="F30">
         <v>23</v>
       </c>
-      <c r="G30">
+      <c r="G30" s="3">
         <v>120</v>
       </c>
-      <c r="H30">
+      <c r="H30" s="3" t="str">
         <f>F30*G30</f>
-        <v>2760</v>
+        <v>$2,760.00</v>
       </c>
       <c r="I30" t="s">
         <v>18</v>
@@ -1357,7 +1545,7 @@
       <c r="A31">
         <v>1030</v>
       </c>
-      <c r="B31" s="1">
+      <c r="B31" s="2">
         <v>45498</v>
       </c>
       <c r="C31" t="s">
@@ -1372,12 +1560,12 @@
       <c r="F31">
         <v>3</v>
       </c>
-      <c r="G31">
+      <c r="G31" s="3">
         <v>120</v>
       </c>
-      <c r="H31">
+      <c r="H31" s="3" t="str">
         <f>F31*G31</f>
-        <v>360</v>
+        <v>$360.00</v>
       </c>
       <c r="I31" t="s">
         <v>16</v>
@@ -1387,7 +1575,7 @@
       <c r="A32">
         <v>1031</v>
       </c>
-      <c r="B32" s="1">
+      <c r="B32" s="2">
         <v>45507</v>
       </c>
       <c r="C32" t="s">
@@ -1402,12 +1590,12 @@
       <c r="F32">
         <v>19</v>
       </c>
-      <c r="G32">
+      <c r="G32" s="3">
         <v>19.99</v>
       </c>
-      <c r="H32">
+      <c r="H32" s="3" t="str">
         <f>F32*G32</f>
-        <v>379.81</v>
+        <v>$379.81</v>
       </c>
       <c r="I32" t="s">
         <v>18</v>
@@ -1417,7 +1605,7 @@
       <c r="A33">
         <v>1032</v>
       </c>
-      <c r="B33" s="1">
+      <c r="B33" s="2">
         <v>45514</v>
       </c>
       <c r="C33" t="s">
@@ -1432,12 +1620,12 @@
       <c r="F33">
         <v>9</v>
       </c>
-      <c r="G33">
+      <c r="G33" s="3">
         <v>120</v>
       </c>
-      <c r="H33">
+      <c r="H33" s="3" t="str">
         <f>F33*G33</f>
-        <v>1080</v>
+        <v>$1,080.00</v>
       </c>
       <c r="I33" t="s">
         <v>18</v>
@@ -1447,7 +1635,7 @@
       <c r="A34">
         <v>1033</v>
       </c>
-      <c r="B34" s="1">
+      <c r="B34" s="2">
         <v>45519</v>
       </c>
       <c r="C34" t="s">
@@ -1462,12 +1650,12 @@
       <c r="F34">
         <v>26</v>
       </c>
-      <c r="G34">
+      <c r="G34" s="3">
         <v>7.25</v>
       </c>
-      <c r="H34">
+      <c r="H34" s="3" t="str">
         <f>F34*G34</f>
-        <v>188.5</v>
+        <v>$188.50</v>
       </c>
       <c r="I34" t="s">
         <v>12</v>
@@ -1477,7 +1665,7 @@
       <c r="A35">
         <v>1034</v>
       </c>
-      <c r="B35" s="1">
+      <c r="B35" s="2">
         <v>45528</v>
       </c>
       <c r="C35" t="s">
@@ -1492,12 +1680,12 @@
       <c r="F35">
         <v>13</v>
       </c>
-      <c r="G35">
+      <c r="G35" s="3">
         <v>42</v>
       </c>
-      <c r="H35">
+      <c r="H35" s="3" t="str">
         <f>F35*G35</f>
-        <v>546</v>
+        <v>$546.00</v>
       </c>
       <c r="I35" t="s">
         <v>16</v>
@@ -1507,7 +1695,7 @@
       <c r="A36">
         <v>1035</v>
       </c>
-      <c r="B36" s="1">
+      <c r="B36" s="2">
         <v>45533</v>
       </c>
       <c r="C36" t="s">
@@ -1522,12 +1710,12 @@
       <c r="F36">
         <v>20</v>
       </c>
-      <c r="G36">
+      <c r="G36" s="3">
         <v>7.25</v>
       </c>
-      <c r="H36">
+      <c r="H36" s="3" t="str">
         <f>F36*G36</f>
-        <v>145</v>
+        <v>$145.00</v>
       </c>
       <c r="I36" t="s">
         <v>12</v>
@@ -1537,7 +1725,7 @@
       <c r="A37">
         <v>1036</v>
       </c>
-      <c r="B37" s="1">
+      <c r="B37" s="2">
         <v>45541</v>
       </c>
       <c r="C37" t="s">
@@ -1552,12 +1740,12 @@
       <c r="F37">
         <v>1</v>
       </c>
-      <c r="G37">
+      <c r="G37" s="3">
         <v>120</v>
       </c>
-      <c r="H37">
+      <c r="H37" s="3" t="str">
         <f>F37*G37</f>
-        <v>120</v>
+        <v>$120.00</v>
       </c>
       <c r="I37" t="s">
         <v>16</v>
@@ -1567,7 +1755,7 @@
       <c r="A38">
         <v>1037</v>
       </c>
-      <c r="B38" s="1">
+      <c r="B38" s="2">
         <v>45548</v>
       </c>
       <c r="C38" t="s">
@@ -1582,12 +1770,12 @@
       <c r="F38">
         <v>27</v>
       </c>
-      <c r="G38">
+      <c r="G38" s="3">
         <v>120</v>
       </c>
-      <c r="H38">
+      <c r="H38" s="3" t="str">
         <f>F38*G38</f>
-        <v>3240</v>
+        <v>$3,240.00</v>
       </c>
       <c r="I38" t="s">
         <v>12</v>
@@ -1597,7 +1785,7 @@
       <c r="A39">
         <v>1038</v>
       </c>
-      <c r="B39" s="1">
+      <c r="B39" s="2">
         <v>45554</v>
       </c>
       <c r="C39" t="s">
@@ -1612,12 +1800,12 @@
       <c r="F39">
         <v>1</v>
       </c>
-      <c r="G39">
+      <c r="G39" s="3">
         <v>42</v>
       </c>
-      <c r="H39">
+      <c r="H39" s="3" t="str">
         <f>F39*G39</f>
-        <v>42</v>
+        <v>$42.00</v>
       </c>
       <c r="I39" t="s">
         <v>12</v>
@@ -1627,7 +1815,7 @@
       <c r="A40">
         <v>1039</v>
       </c>
-      <c r="B40" s="1">
+      <c r="B40" s="2">
         <v>45560</v>
       </c>
       <c r="C40" t="s">
@@ -1642,12 +1830,12 @@
       <c r="F40">
         <v>20</v>
       </c>
-      <c r="G40">
+      <c r="G40" s="3">
         <v>7.25</v>
       </c>
-      <c r="H40">
+      <c r="H40" s="3" t="str">
         <f>F40*G40</f>
-        <v>145</v>
+        <v>$145.00</v>
       </c>
       <c r="I40" t="s">
         <v>12</v>
@@ -1657,7 +1845,7 @@
       <c r="A41">
         <v>1040</v>
       </c>
-      <c r="B41" s="1">
+      <c r="B41" s="2">
         <v>45569</v>
       </c>
       <c r="C41" t="s">
@@ -1672,12 +1860,12 @@
       <c r="F41">
         <v>29</v>
       </c>
-      <c r="G41">
+      <c r="G41" s="3">
         <v>19.99</v>
       </c>
-      <c r="H41">
+      <c r="H41" s="3" t="str">
         <f>F41*G41</f>
-        <v>579.71</v>
+        <v>$579.71</v>
       </c>
       <c r="I41" t="s">
         <v>12</v>
@@ -1687,7 +1875,7 @@
       <c r="A42">
         <v>1041</v>
       </c>
-      <c r="B42" s="1">
+      <c r="B42" s="2">
         <v>45578</v>
       </c>
       <c r="C42" t="s">
@@ -1702,12 +1890,12 @@
       <c r="F42">
         <v>18</v>
       </c>
-      <c r="G42">
+      <c r="G42" s="3">
         <v>3.5</v>
       </c>
-      <c r="H42">
+      <c r="H42" s="3" t="str">
         <f>F42*G42</f>
-        <v>63</v>
+        <v>$63.00</v>
       </c>
       <c r="I42" t="s">
         <v>12</v>
@@ -1717,7 +1905,7 @@
       <c r="A43">
         <v>1042</v>
       </c>
-      <c r="B43" s="1">
+      <c r="B43" s="2">
         <v>45583</v>
       </c>
       <c r="C43" t="s">
@@ -1732,12 +1920,12 @@
       <c r="F43">
         <v>1</v>
       </c>
-      <c r="G43">
+      <c r="G43" s="3">
         <v>19.99</v>
       </c>
-      <c r="H43">
+      <c r="H43" s="3" t="str">
         <f>F43*G43</f>
-        <v>19.99</v>
+        <v>$19.99</v>
       </c>
       <c r="I43" t="s">
         <v>18</v>
@@ -1747,7 +1935,7 @@
       <c r="A44">
         <v>1043</v>
       </c>
-      <c r="B44" s="1">
+      <c r="B44" s="2">
         <v>45592</v>
       </c>
       <c r="C44" t="s">
@@ -1762,12 +1950,12 @@
       <c r="F44">
         <v>8</v>
       </c>
-      <c r="G44">
+      <c r="G44" s="3">
         <v>7.25</v>
       </c>
-      <c r="H44">
+      <c r="H44" s="3" t="str">
         <f>F44*G44</f>
-        <v>58</v>
+        <v>$58.00</v>
       </c>
       <c r="I44" t="s">
         <v>12</v>
@@ -1777,7 +1965,7 @@
       <c r="A45">
         <v>1044</v>
       </c>
-      <c r="B45" s="1">
+      <c r="B45" s="2">
         <v>45596</v>
       </c>
       <c r="C45" t="s">
@@ -1792,12 +1980,12 @@
       <c r="F45">
         <v>36</v>
       </c>
-      <c r="G45">
+      <c r="G45" s="3">
         <v>7.25</v>
       </c>
-      <c r="H45">
+      <c r="H45" s="3" t="str">
         <f>F45*G45</f>
-        <v>261</v>
+        <v>$261.00</v>
       </c>
       <c r="I45" t="s">
         <v>12</v>
@@ -1807,7 +1995,7 @@
       <c r="A46">
         <v>1045</v>
       </c>
-      <c r="B46" s="1">
+      <c r="B46" s="2">
         <v>45604</v>
       </c>
       <c r="C46" t="s">
@@ -1822,12 +2010,12 @@
       <c r="F46">
         <v>29</v>
       </c>
-      <c r="G46">
+      <c r="G46" s="3">
         <v>7.25</v>
       </c>
-      <c r="H46">
+      <c r="H46" s="3" t="str">
         <f>F46*G46</f>
-        <v>210.25</v>
+        <v>$210.25</v>
       </c>
       <c r="I46" t="s">
         <v>16</v>
@@ -1837,7 +2025,7 @@
       <c r="A47">
         <v>1046</v>
       </c>
-      <c r="B47" s="1">
+      <c r="B47" s="2">
         <v>45610</v>
       </c>
       <c r="C47" t="s">
@@ -1852,12 +2040,12 @@
       <c r="F47">
         <v>35</v>
       </c>
-      <c r="G47">
+      <c r="G47" s="3">
         <v>19.99</v>
       </c>
-      <c r="H47">
+      <c r="H47" s="3" t="str">
         <f>F47*G47</f>
-        <v>699.65</v>
+        <v>$699.65</v>
       </c>
       <c r="I47" t="s">
         <v>16</v>
@@ -1867,7 +2055,7 @@
       <c r="A48">
         <v>1047</v>
       </c>
-      <c r="B48" s="1">
+      <c r="B48" s="2">
         <v>45619</v>
       </c>
       <c r="C48" t="s">
@@ -1882,12 +2070,12 @@
       <c r="F48">
         <v>34</v>
       </c>
-      <c r="G48">
+      <c r="G48" s="3">
         <v>3.5</v>
       </c>
-      <c r="H48">
+      <c r="H48" s="3" t="str">
         <f>F48*G48</f>
-        <v>119</v>
+        <v>$119.00</v>
       </c>
       <c r="I48" t="s">
         <v>18</v>
@@ -1897,7 +2085,7 @@
       <c r="A49">
         <v>1048</v>
       </c>
-      <c r="B49" s="1">
+      <c r="B49" s="2">
         <v>45623</v>
       </c>
       <c r="C49" t="s">
@@ -1912,12 +2100,12 @@
       <c r="F49">
         <v>25</v>
       </c>
-      <c r="G49">
+      <c r="G49" s="3">
         <v>19.99</v>
       </c>
-      <c r="H49">
+      <c r="H49" s="3" t="str">
         <f>F49*G49</f>
-        <v>499.75</v>
+        <v>$499.75</v>
       </c>
       <c r="I49" t="s">
         <v>16</v>
@@ -1939,16 +2127,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>28</v>
       </c>
     </row>
@@ -1956,85 +2144,85 @@
       <c r="A2" t="s">
         <v>9</v>
       </c>
-      <c r="B2">
+      <c r="B2" s="3" t="str">
         <f>SUMIF(Orders!C$2:C$49,A2,Orders!H$2:H$49)</f>
-        <v>9439.3</v>
+        <v>$9,439.30</v>
       </c>
       <c r="C2">
         <f>COUNTIF(Orders!C$2:C$49,A2)</f>
         <v>10</v>
       </c>
-      <c r="D2">
+      <c r="D2" s="3" t="str">
         <f>ROUND(B2/C2,2)</f>
-        <v>943.93</v>
+        <v>$943.93</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" t="s">
         <v>23</v>
       </c>
-      <c r="B3">
+      <c r="B3" s="3" t="str">
         <f>SUMIF(Orders!C$2:C$49,A3,Orders!H$2:H$49)</f>
-        <v>6570.89</v>
+        <v>$6,570.89</v>
       </c>
       <c r="C3">
         <f>COUNTIF(Orders!C$2:C$49,A3)</f>
         <v>11</v>
       </c>
-      <c r="D3">
+      <c r="D3" s="3" t="str">
         <f>ROUND(B3/C3,2)</f>
-        <v>597.35</v>
+        <v>$597.35</v>
       </c>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" t="s">
         <v>13</v>
       </c>
-      <c r="B4">
+      <c r="B4" s="3" t="str">
         <f>SUMIF(Orders!C$2:C$49,A4,Orders!H$2:H$49)</f>
-        <v>7837</v>
+        <v>$7,837.00</v>
       </c>
       <c r="C4">
         <f>COUNTIF(Orders!C$2:C$49,A4)</f>
         <v>15</v>
       </c>
-      <c r="D4">
+      <c r="D4" s="3" t="str">
         <f>ROUND(B4/C4,2)</f>
-        <v>522.47</v>
+        <v>$522.47</v>
       </c>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" t="s">
         <v>19</v>
       </c>
-      <c r="B5">
+      <c r="B5" s="3" t="str">
         <f>SUMIF(Orders!C$2:C$49,A5,Orders!H$2:H$49)</f>
-        <v>11192.7</v>
+        <v>$11,192.70</v>
       </c>
       <c r="C5">
         <f>COUNTIF(Orders!C$2:C$49,A5)</f>
         <v>12</v>
       </c>
-      <c r="D5">
+      <c r="D5" s="3" t="str">
         <f>ROUND(B5/C5,2)</f>
-        <v>932.73</v>
+        <v>$932.73</v>
       </c>
     </row>
     <row r="6" spans="1:4">
-      <c r="A6" t="s">
+      <c r="A6" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="B6">
+      <c r="B6" s="5" t="str">
         <f>SUM(B2:B5)</f>
-        <v>35039.89</v>
-      </c>
-      <c r="C6">
+        <v>$35,039.89</v>
+      </c>
+      <c r="C6" s="4">
         <f>SUM(C2:C5)</f>
         <v>48</v>
       </c>
-      <c r="D6">
+      <c r="D6" s="5" t="str">
         <f>ROUND(B6/C6,2)</f>
-        <v>730</v>
+        <v>$730.00</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -2048,5 +2236,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>